<commit_message>
feat: add API health check functionality with error tracking
- Implemented ApiHealthCard component for testing external API connections.
- Created route for API health checks, including GET and POST methods.
- Added functions to record and clear API errors in the database.
- Integrated employee lookup and email sending tests in the health check process.

Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/test-import-errors.xlsx
+++ b/test-import-errors.xlsx
@@ -948,10 +948,10 @@
         <v>46</v>
       </c>
       <c r="F2" s="2">
-        <v>32</v>
+        <v>80</v>
       </c>
       <c r="G2" s="2">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="H2" s="2">
         <v>1</v>
@@ -1204,10 +1204,10 @@
         <v>6</v>
       </c>
       <c r="F10">
-        <v>27</v>
+        <v>69</v>
       </c>
       <c r="G10">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="H10">
         <v>1</v>
@@ -1236,10 +1236,10 @@
         <v>6</v>
       </c>
       <c r="F11">
-        <v>32</v>
+        <v>80</v>
       </c>
       <c r="G11">
-        <v>40</v>
+        <v>91</v>
       </c>
       <c r="H11">
         <v>1</v>
@@ -1268,10 +1268,10 @@
         <v>6</v>
       </c>
       <c r="F12">
-        <v>32</v>
+        <v>80</v>
       </c>
       <c r="G12">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="H12">
         <v>10</v>
@@ -1300,10 +1300,10 @@
         <v>6</v>
       </c>
       <c r="F13">
-        <v>32</v>
+        <v>80</v>
       </c>
       <c r="G13">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="H13">
         <v>1</v>
@@ -1364,10 +1364,10 @@
         <v>46</v>
       </c>
       <c r="F15">
-        <v>32</v>
+        <v>80</v>
       </c>
       <c r="G15">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="H15">
         <v>1</v>
@@ -1428,10 +1428,10 @@
         <v>6</v>
       </c>
       <c r="F17">
-        <v>34</v>
+        <v>85</v>
       </c>
       <c r="G17">
-        <v>32</v>
+        <v>80</v>
       </c>
       <c r="H17">
         <v>1</v>

</xml_diff>